<commit_message>
Analysis with 100 datasets per model per type
</commit_message>
<xml_diff>
--- a/comparison_metrics/parafit_summary_cosp.xlsx
+++ b/comparison_metrics/parafit_summary_cosp.xlsx
@@ -1,76 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriele/synthetic_cophylo/comparison_metrics/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0FDB80-0125-354A-89E3-05ED40F49A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="3400" windowWidth="34560" windowHeight="20060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>model</t>
-  </si>
-  <si>
-    <t>mean_stat</t>
-  </si>
-  <si>
-    <t>std_stat</t>
-  </si>
-  <si>
-    <t>num_datasets</t>
-  </si>
-  <si>
-    <t>num_significant</t>
-  </si>
-  <si>
-    <t>pct_significant</t>
-  </si>
-  <si>
-    <t>Alcala_Cosp</t>
-  </si>
-  <si>
-    <t>Coala_Cosp</t>
-  </si>
-  <si>
-    <t>Treeducken_Cosp</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -85,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -408,134 +419,111 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{4E13F0C5-5EA7-AD40-A16C-C75AEA9E3B60}">
-  <we:reference id="026e7b2b-fa4d-4fe0-bf3b-b965f6f25bee" version="1.0.0.78" store="EXCatalog" storeType="EXCatalog"/>
-  <we:alternateReferences>
-    <we:reference id="WA200000565" version="1.0.0.78" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties/>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-  <we:extLst>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
-      <we:containsCustomFunctions/>
-    </a:ext>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
-      <we:customFunctionIdList>
-        <we:customFunctionIds>RDP.Data</we:customFunctionIds>
-        <we:customFunctionIds>RDP.Price</we:customFunctionIds>
-        <we:customFunctionIds>RDP.HistoricalPricing</we:customFunctionIds>
-        <we:customFunctionIds>RDP.Analytics</we:customFunctionIds>
-        <we:customFunctionIds>RDP.Search</we:customFunctionIds>
-        <we:customFunctionIds>RDP.Now</we:customFunctionIds>
-        <we:customFunctionIds>RDP.Today</we:customFunctionIds>
-        <we:customFunctionIds>RDP.Aggregate</we:customFunctionIds>
-      </we:customFunctionIdList>
-    </a:ext>
-  </we:extLst>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>mean_stat</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>std_stat</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>num_datasets</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>num_significant</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>pct_significant</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>16912.900000000001</v>
-      </c>
-      <c r="C2">
-        <v>23716.32</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Alcala_Cosp</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4119.81</v>
+      </c>
+      <c r="C2" t="n">
+        <v>12080.01</v>
+      </c>
+      <c r="D2" t="n">
+        <v>41</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>17.07</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>29487848.43</v>
-      </c>
-      <c r="C3">
-        <v>34774124.200000003</v>
-      </c>
-      <c r="D3">
-        <v>10</v>
-      </c>
-      <c r="E3">
-        <v>10</v>
-      </c>
-      <c r="F3">
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Coala_Cosp</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>111041776.41</v>
+      </c>
+      <c r="C3" t="n">
+        <v>320861702.52</v>
+      </c>
+      <c r="D3" t="n">
+        <v>94</v>
+      </c>
+      <c r="E3" t="n">
+        <v>94</v>
+      </c>
+      <c r="F3" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4">
-        <v>2780.22</v>
-      </c>
-      <c r="C4">
-        <v>5884.39</v>
-      </c>
-      <c r="D4">
-        <v>10</v>
-      </c>
-      <c r="E4">
-        <v>9</v>
-      </c>
-      <c r="F4">
-        <v>90</v>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Treeducken_Cosp</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6627.66</v>
+      </c>
+      <c r="C4" t="n">
+        <v>12734.24</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" t="n">
+        <v>89</v>
+      </c>
+      <c r="F4" t="n">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Analysis on 500 Dataset each
</commit_message>
<xml_diff>
--- a/comparison_metrics/parafit_summary_cosp.xlsx
+++ b/comparison_metrics/parafit_summary_cosp.xlsx
@@ -467,19 +467,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4119.81</v>
+        <v>11385.47</v>
       </c>
       <c r="C2" t="n">
-        <v>12080.01</v>
+        <v>66293.61</v>
       </c>
       <c r="D2" t="n">
-        <v>41</v>
+        <v>191</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="F2" t="n">
-        <v>17.07</v>
+        <v>29.84</v>
       </c>
     </row>
     <row r="3">
@@ -489,19 +489,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>111041776.41</v>
+        <v>114856120.66</v>
       </c>
       <c r="C3" t="n">
-        <v>320861702.52</v>
+        <v>441664692.97</v>
       </c>
       <c r="D3" t="n">
-        <v>94</v>
+        <v>500</v>
       </c>
       <c r="E3" t="n">
-        <v>94</v>
+        <v>495</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4">
@@ -520,10 +520,10 @@
         <v>23</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F4" t="n">
-        <v>56.52</v>
+        <v>65.22</v>
       </c>
     </row>
     <row r="5">
@@ -533,19 +533,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6627.66</v>
+        <v>4831.76</v>
       </c>
       <c r="C5" t="n">
-        <v>12734.24</v>
+        <v>11404.17</v>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>497</v>
       </c>
       <c r="E5" t="n">
-        <v>88</v>
+        <v>426</v>
       </c>
       <c r="F5" t="n">
-        <v>88</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Some adjustmets to comparison metrics
</commit_message>
<xml_diff>
--- a/comparison_metrics/parafit_summary_cosp.xlsx
+++ b/comparison_metrics/parafit_summary_cosp.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,76 +476,98 @@
         <v>191</v>
       </c>
       <c r="E2" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>29.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Coala_Cosp</t>
+          <t>Asymmetree_Cosp</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>114856120.66</v>
+        <v>16350.03</v>
       </c>
       <c r="C3" t="n">
-        <v>441664692.97</v>
+        <v>15027.43</v>
       </c>
       <c r="D3" t="n">
         <v>500</v>
       </c>
       <c r="E3" t="n">
-        <v>495</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Real_Data</t>
+          <t>Coala_Cosp</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15807.72</v>
+        <v>114856120.66</v>
       </c>
       <c r="C4" t="n">
-        <v>21682.83</v>
+        <v>441664692.97</v>
       </c>
       <c r="D4" t="n">
-        <v>23</v>
+        <v>500</v>
       </c>
       <c r="E4" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>65.22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>205038484.64</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1164019159.73</v>
+      </c>
+      <c r="D5" t="n">
+        <v>33</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
           <t>Treeducken_Cosp</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
         <v>4831.76</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C6" t="n">
         <v>11404.17</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D6" t="n">
         <v>497</v>
       </c>
-      <c r="E5" t="n">
-        <v>426</v>
-      </c>
-      <c r="F5" t="n">
-        <v>85.70999999999999</v>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>